<commit_message>
changed god dragon to just god
</commit_message>
<xml_diff>
--- a/DV3_breed data.xlsx
+++ b/DV3_breed data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tky12\OneDrive\桌面\DV3 breed calculator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5483270B-5310-45C4-931D-7A3762DA8DD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64D4B24B-B1F3-4FC8-B24A-ECA2B1E11B68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5448" yWindow="1344" windowWidth="14160" windowHeight="9120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Base Hatching Time" sheetId="1" r:id="rId1"/>
@@ -197,9 +197,6 @@
     <t>Goblin</t>
   </si>
   <si>
-    <t>God Dragon</t>
-  </si>
-  <si>
     <t>Goldie</t>
   </si>
   <si>
@@ -441,6 +438,9 @@
   </si>
   <si>
     <t>Legendary</t>
+  </si>
+  <si>
+    <t>God</t>
   </si>
 </sst>
 </file>
@@ -884,7 +884,7 @@
         <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J1" t="s">
         <v>9</v>
@@ -899,16 +899,16 @@
         <v>12</v>
       </c>
       <c r="N1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="O1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="P1" t="s">
         <v>13</v>
       </c>
       <c r="Q1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
@@ -922,10 +922,10 @@
         <v>1</v>
       </c>
       <c r="P2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.3">
@@ -939,10 +939,10 @@
         <v>1</v>
       </c>
       <c r="P3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="R3" t="s">
         <v>16</v>
@@ -960,15 +960,15 @@
         <v>1</v>
       </c>
       <c r="P4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B5">
         <f>22.5/60</f>
@@ -978,15 +978,15 @@
         <v>1</v>
       </c>
       <c r="P5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -995,15 +995,15 @@
         <v>1</v>
       </c>
       <c r="P6" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B7">
         <v>2</v>
@@ -1018,10 +1018,10 @@
         <v>1</v>
       </c>
       <c r="P7" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q7" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.3">
@@ -1038,15 +1038,15 @@
         <v>1</v>
       </c>
       <c r="P8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B9">
         <v>2</v>
@@ -1058,21 +1058,21 @@
         <v>1</v>
       </c>
       <c r="P9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B10">
         <v>2</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -1084,10 +1084,10 @@
         <v>4</v>
       </c>
       <c r="P10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.3">
@@ -1108,15 +1108,15 @@
         <v>1</v>
       </c>
       <c r="P11" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q11" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B12">
         <v>2.25</v>
@@ -1131,10 +1131,10 @@
         <v>1</v>
       </c>
       <c r="P12" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q12" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.3">
@@ -1148,15 +1148,15 @@
         <v>1</v>
       </c>
       <c r="P13" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B14">
         <v>2.5</v>
@@ -1171,15 +1171,15 @@
         <v>1</v>
       </c>
       <c r="P14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B15">
         <v>2.5</v>
@@ -1194,15 +1194,15 @@
         <v>1</v>
       </c>
       <c r="P15" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q15" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B16">
         <v>2.5</v>
@@ -1217,10 +1217,10 @@
         <v>1</v>
       </c>
       <c r="P16" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q16" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.3">
@@ -1240,15 +1240,15 @@
         <v>1</v>
       </c>
       <c r="P17" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q17" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B18">
         <v>2.75</v>
@@ -1263,15 +1263,15 @@
         <v>1</v>
       </c>
       <c r="P18" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q18" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B19">
         <v>3</v>
@@ -1286,10 +1286,10 @@
         <v>1</v>
       </c>
       <c r="P19" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q19" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.3">
@@ -1300,7 +1300,7 @@
         <v>3.25</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D20">
         <v>1</v>
@@ -1312,15 +1312,15 @@
         <v>4</v>
       </c>
       <c r="P20" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q20" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B21">
         <v>3.25</v>
@@ -1335,10 +1335,10 @@
         <v>1</v>
       </c>
       <c r="P21" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q21" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.3">
@@ -1353,15 +1353,15 @@
         <v>1</v>
       </c>
       <c r="P22" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q22" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B23">
         <v>3.75</v>
@@ -1376,15 +1376,15 @@
         <v>1</v>
       </c>
       <c r="P23" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q23" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B24">
         <v>4.25</v>
@@ -1399,15 +1399,15 @@
         <v>1</v>
       </c>
       <c r="P24" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q24" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B25">
         <v>4.375</v>
@@ -1422,15 +1422,15 @@
         <v>1</v>
       </c>
       <c r="P25" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q25" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B26">
         <v>4.625</v>
@@ -1445,15 +1445,15 @@
         <v>1</v>
       </c>
       <c r="P26" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q26" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B27">
         <v>5.25</v>
@@ -1468,15 +1468,15 @@
         <v>1</v>
       </c>
       <c r="P27" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q27" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="28" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B28">
         <v>5.5</v>
@@ -1491,15 +1491,15 @@
         <v>1</v>
       </c>
       <c r="P28" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q28" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B29">
         <v>5.5</v>
@@ -1514,15 +1514,15 @@
         <v>1</v>
       </c>
       <c r="P29" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q29" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B30">
         <v>5.5</v>
@@ -1537,15 +1537,15 @@
         <v>1</v>
       </c>
       <c r="P30" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q30" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B31">
         <v>6</v>
@@ -1560,21 +1560,21 @@
         <v>1</v>
       </c>
       <c r="P31" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q31" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="32" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B32">
         <v>6.125</v>
       </c>
       <c r="C32" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="H32">
         <v>1</v>
@@ -1583,10 +1583,10 @@
         <v>1</v>
       </c>
       <c r="P32" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q32" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.3">
@@ -1603,15 +1603,15 @@
         <v>1</v>
       </c>
       <c r="P33" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q33" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B34">
         <v>6.25</v>
@@ -1623,15 +1623,15 @@
         <v>1</v>
       </c>
       <c r="P34" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q34" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B35">
         <v>6.5</v>
@@ -1640,21 +1640,21 @@
         <v>1</v>
       </c>
       <c r="P35" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q35" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B36">
         <v>6.5</v>
       </c>
       <c r="C36" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="I36">
         <v>1</v>
@@ -1663,10 +1663,10 @@
         <v>1</v>
       </c>
       <c r="P36" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q36" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.3">
@@ -1686,15 +1686,15 @@
         <v>1</v>
       </c>
       <c r="P37" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q37" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="38" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B38">
         <v>6.75</v>
@@ -1709,15 +1709,15 @@
         <v>1</v>
       </c>
       <c r="P38" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q38" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="39" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B39">
         <v>6.75</v>
@@ -1732,15 +1732,15 @@
         <v>1</v>
       </c>
       <c r="P39" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q39" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="40" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B40">
         <v>6.75</v>
@@ -1755,10 +1755,10 @@
         <v>1</v>
       </c>
       <c r="P40" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q40" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="41" spans="1:17" x14ac:dyDescent="0.3">
@@ -1778,15 +1778,15 @@
         <v>1</v>
       </c>
       <c r="P41" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q41" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="42" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B42">
         <v>6.875</v>
@@ -1801,15 +1801,15 @@
         <v>1</v>
       </c>
       <c r="P42" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q42" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="43" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B43">
         <v>6.875</v>
@@ -1824,15 +1824,15 @@
         <v>1</v>
       </c>
       <c r="P43" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q43" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="44" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B44">
         <v>6.875</v>
@@ -1847,15 +1847,15 @@
         <v>1</v>
       </c>
       <c r="P44" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q44" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="45" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B45">
         <v>7</v>
@@ -1864,10 +1864,10 @@
         <v>1</v>
       </c>
       <c r="P45" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q45" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="46" spans="1:17" x14ac:dyDescent="0.3">
@@ -1887,15 +1887,15 @@
         <v>1</v>
       </c>
       <c r="P46" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q46" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="47" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B47">
         <v>7</v>
@@ -1910,15 +1910,15 @@
         <v>1</v>
       </c>
       <c r="P47" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q47" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="48" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B48">
         <v>7</v>
@@ -1933,15 +1933,15 @@
         <v>1</v>
       </c>
       <c r="P48" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q48" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="49" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B49">
         <v>7.125</v>
@@ -1956,15 +1956,15 @@
         <v>1</v>
       </c>
       <c r="P49" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q49" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="50" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B50">
         <v>7.125</v>
@@ -1979,10 +1979,10 @@
         <v>1</v>
       </c>
       <c r="P50" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q50" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="51" spans="1:17" x14ac:dyDescent="0.3">
@@ -1999,10 +1999,10 @@
         <v>1</v>
       </c>
       <c r="P51" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q51" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="52" spans="1:17" x14ac:dyDescent="0.3">
@@ -2013,21 +2013,21 @@
         <v>7.25</v>
       </c>
       <c r="P52" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q52" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="53" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B53">
         <v>7.25</v>
       </c>
       <c r="C53" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E53">
         <v>1</v>
@@ -2036,10 +2036,10 @@
         <v>1</v>
       </c>
       <c r="P53" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q53" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="54" spans="1:17" x14ac:dyDescent="0.3">
@@ -2059,10 +2059,10 @@
         <v>1</v>
       </c>
       <c r="P54" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q54" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="55" spans="1:17" x14ac:dyDescent="0.3">
@@ -2082,15 +2082,15 @@
         <v>1</v>
       </c>
       <c r="P55" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q55" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="56" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B56">
         <v>7.25</v>
@@ -2105,15 +2105,15 @@
         <v>1</v>
       </c>
       <c r="P56" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q56" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="57" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B57">
         <v>7.25</v>
@@ -2128,15 +2128,15 @@
         <v>1</v>
       </c>
       <c r="P57" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q57" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="58" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B58">
         <v>7.25</v>
@@ -2151,21 +2151,21 @@
         <v>1</v>
       </c>
       <c r="P58" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q58" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="59" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B59">
         <v>7.25</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E59">
         <v>1</v>
@@ -2177,10 +2177,10 @@
         <v>4</v>
       </c>
       <c r="P59" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q59" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="60" spans="1:17" x14ac:dyDescent="0.3">
@@ -2191,7 +2191,7 @@
         <v>7.375</v>
       </c>
       <c r="C60" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F60">
         <v>1</v>
@@ -2200,15 +2200,15 @@
         <v>1</v>
       </c>
       <c r="P60" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q60" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="61" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B61">
         <v>7.375</v>
@@ -2220,15 +2220,15 @@
         <v>1</v>
       </c>
       <c r="P61" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q61" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="62" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B62">
         <v>7.375</v>
@@ -2243,15 +2243,15 @@
         <v>1</v>
       </c>
       <c r="P62" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q62" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="63" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B63">
         <v>7.375</v>
@@ -2266,15 +2266,15 @@
         <v>1</v>
       </c>
       <c r="P63" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q63" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="64" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B64">
         <v>7.375</v>
@@ -2289,15 +2289,15 @@
         <v>1</v>
       </c>
       <c r="P64" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q64" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="65" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B65">
         <v>7.375</v>
@@ -2312,10 +2312,10 @@
         <v>1</v>
       </c>
       <c r="P65" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q65" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="66" spans="1:17" x14ac:dyDescent="0.3">
@@ -2335,15 +2335,15 @@
         <v>1</v>
       </c>
       <c r="P66" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q66" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="67" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B67">
         <v>7.5</v>
@@ -2358,15 +2358,15 @@
         <v>1</v>
       </c>
       <c r="P67" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q67" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="68" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B68">
         <v>7.5</v>
@@ -2381,21 +2381,21 @@
         <v>1</v>
       </c>
       <c r="P68" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q68" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="69" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B69">
         <v>7.6749999999999998</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F69">
         <v>1</v>
@@ -2404,10 +2404,10 @@
         <v>1</v>
       </c>
       <c r="P69" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q69" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="70" spans="1:17" x14ac:dyDescent="0.3">
@@ -2424,10 +2424,10 @@
         <v>1</v>
       </c>
       <c r="P70" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q70" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="71" spans="1:17" x14ac:dyDescent="0.3">
@@ -2447,15 +2447,15 @@
         <v>1</v>
       </c>
       <c r="P71" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q71" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="72" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B72">
         <v>7.75</v>
@@ -2470,15 +2470,15 @@
         <v>1</v>
       </c>
       <c r="P72" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q72" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="73" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B73">
         <v>7.75</v>
@@ -2493,10 +2493,10 @@
         <v>1</v>
       </c>
       <c r="P73" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q73" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="74" spans="1:17" x14ac:dyDescent="0.3">
@@ -2507,7 +2507,7 @@
         <v>8</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F74">
         <v>1</v>
@@ -2516,10 +2516,10 @@
         <v>1</v>
       </c>
       <c r="P74" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q74" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="75" spans="1:17" x14ac:dyDescent="0.3">
@@ -2530,7 +2530,7 @@
         <v>8</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F75">
         <v>1</v>
@@ -2539,21 +2539,21 @@
         <v>1</v>
       </c>
       <c r="P75" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q75" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="76" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B76">
         <v>8</v>
       </c>
       <c r="C76" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="J76">
         <v>1</v>
@@ -2562,21 +2562,21 @@
         <v>1</v>
       </c>
       <c r="P76" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q76" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="77" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B77">
         <v>8</v>
       </c>
       <c r="C77" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K77">
         <v>1</v>
@@ -2588,10 +2588,10 @@
         <v>4</v>
       </c>
       <c r="P77" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q77" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="78" spans="1:17" x14ac:dyDescent="0.3">
@@ -2602,7 +2602,7 @@
         <v>8.25</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G78">
         <v>1</v>
@@ -2611,10 +2611,10 @@
         <v>1</v>
       </c>
       <c r="P78" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q78" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="79" spans="1:17" x14ac:dyDescent="0.3">
@@ -2625,7 +2625,7 @@
         <v>8.25</v>
       </c>
       <c r="C79" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D79">
         <v>1</v>
@@ -2637,10 +2637,10 @@
         <v>4</v>
       </c>
       <c r="P79" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q79" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="80" spans="1:17" x14ac:dyDescent="0.3">
@@ -2651,7 +2651,7 @@
         <v>8.25</v>
       </c>
       <c r="C80" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G80">
         <v>1</v>
@@ -2660,15 +2660,15 @@
         <v>1</v>
       </c>
       <c r="P80" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q80" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="81" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B81">
         <v>8.25</v>
@@ -2680,15 +2680,15 @@
         <v>1</v>
       </c>
       <c r="P81" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q81" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="82" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B82">
         <v>8.25</v>
@@ -2700,15 +2700,15 @@
         <v>1</v>
       </c>
       <c r="P82" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q82" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="83" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B83">
         <v>8.25</v>
@@ -2723,10 +2723,10 @@
         <v>1</v>
       </c>
       <c r="P83" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q83" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="84" spans="1:17" x14ac:dyDescent="0.3">
@@ -2737,7 +2737,7 @@
         <v>8.5</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K84">
         <v>1</v>
@@ -2746,15 +2746,15 @@
         <v>1</v>
       </c>
       <c r="P84" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q84" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="85" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B85">
         <v>8.5</v>
@@ -2769,21 +2769,21 @@
         <v>1</v>
       </c>
       <c r="P85" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q85" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="86" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B86">
         <v>9.125</v>
       </c>
       <c r="C86" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G86">
         <v>1</v>
@@ -2795,10 +2795,10 @@
         <v>4</v>
       </c>
       <c r="P86" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q86" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="87" spans="1:17" x14ac:dyDescent="0.3">
@@ -2818,15 +2818,15 @@
         <v>1</v>
       </c>
       <c r="P87" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q87" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="88" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B88">
         <v>9.125</v>
@@ -2841,15 +2841,15 @@
         <v>1</v>
       </c>
       <c r="P88" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q88" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="89" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B89">
         <v>14.25</v>
@@ -2864,21 +2864,21 @@
         <v>1</v>
       </c>
       <c r="P89" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q89" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="90" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B90">
         <v>14.25</v>
       </c>
       <c r="C90" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -2890,21 +2890,21 @@
         <v>1</v>
       </c>
       <c r="P90" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q90" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="91" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B91">
         <v>14.875</v>
       </c>
       <c r="C91" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F91">
         <v>1</v>
@@ -2916,21 +2916,21 @@
         <v>1</v>
       </c>
       <c r="P91" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q91" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="92" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B92">
         <v>15</v>
       </c>
       <c r="C92" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D92">
         <v>1</v>
@@ -2942,21 +2942,21 @@
         <v>1</v>
       </c>
       <c r="P92" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q92" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="93" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B93">
         <v>15.5</v>
       </c>
       <c r="C93" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D93">
         <v>1</v>
@@ -2968,10 +2968,10 @@
         <v>1</v>
       </c>
       <c r="P93" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q93" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="94" spans="1:17" x14ac:dyDescent="0.3">
@@ -2991,21 +2991,21 @@
         <v>1</v>
       </c>
       <c r="P94" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q94" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="95" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B95">
         <v>15.625</v>
       </c>
       <c r="C95" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D95">
         <v>1</v>
@@ -3017,10 +3017,10 @@
         <v>1</v>
       </c>
       <c r="P95" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q95" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="96" spans="1:17" x14ac:dyDescent="0.3">
@@ -3031,7 +3031,7 @@
         <v>15.75</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G96">
         <v>1</v>
@@ -3043,15 +3043,15 @@
         <v>1</v>
       </c>
       <c r="P96" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q96" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="97" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B97">
         <v>16</v>
@@ -3066,10 +3066,10 @@
         <v>1</v>
       </c>
       <c r="P97" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q97" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="98" spans="1:17" x14ac:dyDescent="0.3">
@@ -3089,10 +3089,10 @@
         <v>1</v>
       </c>
       <c r="P98" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q98" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="99" spans="1:17" x14ac:dyDescent="0.3">
@@ -3103,7 +3103,7 @@
         <v>16.625</v>
       </c>
       <c r="C99" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F99">
         <v>1</v>
@@ -3115,10 +3115,10 @@
         <v>1</v>
       </c>
       <c r="P99" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q99" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="100" spans="1:17" x14ac:dyDescent="0.3">
@@ -3138,21 +3138,21 @@
         <v>1</v>
       </c>
       <c r="P100" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q100" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="101" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B101">
         <v>16.75</v>
       </c>
       <c r="C101" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3164,18 +3164,18 @@
         <v>1</v>
       </c>
       <c r="O101" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="P101" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q101" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="102" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B102">
         <v>16.75</v>
@@ -3190,15 +3190,15 @@
         <v>1</v>
       </c>
       <c r="P102" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q102" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="103" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B103">
         <v>16.75</v>
@@ -3213,10 +3213,10 @@
         <v>1</v>
       </c>
       <c r="P103" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q103" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="104" spans="1:17" x14ac:dyDescent="0.3">
@@ -3236,10 +3236,10 @@
         <v>1</v>
       </c>
       <c r="P104" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q104" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="105" spans="1:17" x14ac:dyDescent="0.3">
@@ -3259,24 +3259,24 @@
         <v>1</v>
       </c>
       <c r="P105" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q105" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="106" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B106">
         <v>17</v>
       </c>
       <c r="P106" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q106" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="107" spans="1:17" x14ac:dyDescent="0.3">
@@ -3287,7 +3287,7 @@
         <v>18</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="K107">
         <v>1</v>
@@ -3302,10 +3302,10 @@
         <v>5</v>
       </c>
       <c r="P107" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q107" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="108" spans="1:17" x14ac:dyDescent="0.3">
@@ -3316,7 +3316,7 @@
         <v>18</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F108">
         <v>1</v>
@@ -3331,10 +3331,10 @@
         <v>5</v>
       </c>
       <c r="P108" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q108" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="109" spans="1:17" x14ac:dyDescent="0.3">
@@ -3354,10 +3354,10 @@
         <v>1</v>
       </c>
       <c r="P109" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q109" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="110" spans="1:17" x14ac:dyDescent="0.3">
@@ -3377,15 +3377,15 @@
         <v>1</v>
       </c>
       <c r="P110" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q110" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="111" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B111">
         <v>18</v>
@@ -3400,10 +3400,10 @@
         <v>1</v>
       </c>
       <c r="P111" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q111" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="112" spans="1:17" x14ac:dyDescent="0.3">
@@ -3414,24 +3414,24 @@
         <v>23.5</v>
       </c>
       <c r="P112" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q112" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="113" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>54</v>
+        <v>135</v>
       </c>
       <c r="B113">
         <v>24</v>
       </c>
       <c r="P113" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q113" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
   </sheetData>

</xml_diff>